<commit_message>
added pi motor test
</commit_message>
<xml_diff>
--- a/hardware/Components.xlsx
+++ b/hardware/Components.xlsx
@@ -5,17 +5,17 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adamaxelrod/Library/Mobile Documents/com~apple~CloudDocs/UniBots/UniBots/Hardware/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adamaxelrod/Library/Mobile Documents/com~apple~CloudDocs/UniBots/UniBots/hardware/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E6EA341-979A-1E47-A6FF-16413DF48A5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0ABBCC96-1DE8-7A4A-8184-67044864BC74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{C1DFA535-1927-B64A-ABE0-0E77A41D7358}"/>
+    <workbookView xWindow="-36520" yWindow="1960" windowWidth="28800" windowHeight="17400" xr2:uid="{C1DFA535-1927-B64A-ABE0-0E77A41D7358}"/>
   </bookViews>
   <sheets>
     <sheet name="Components" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -582,7 +582,7 @@
         <v>1</v>
       </c>
       <c r="D6" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
@@ -596,7 +596,7 @@
         <v>1</v>
       </c>
       <c r="D7" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
@@ -610,7 +610,7 @@
         <v>1</v>
       </c>
       <c r="D8" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
@@ -624,7 +624,7 @@
         <v>1</v>
       </c>
       <c r="D9" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
@@ -638,7 +638,7 @@
         <v>1</v>
       </c>
       <c r="D10" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
@@ -652,7 +652,7 @@
         <v>1</v>
       </c>
       <c r="D11" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
@@ -670,7 +670,7 @@
       </c>
       <c r="B14" s="2">
         <f>SUMIF(D2:D11,FALSE,B2:B11)</f>
-        <v>100.16</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>